<commit_message>
[update] update AAL mask
</commit_message>
<xml_diff>
--- a/template/ROI mapping.xlsx
+++ b/template/ROI mapping.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="\\172.30.1.87\storage2\Daesung\PRGNN\template\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{794A7C76-28CD-485E-A2E8-A9D96C73B85F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{45BE5D90-A615-403D-9961-F63D35B15887}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -344,9 +344,6 @@
     <t>6101; 6102</t>
   </si>
   <si>
-    <t>6202; 6203</t>
-  </si>
-  <si>
     <t>6211; 6212</t>
   </si>
   <si>
@@ -426,6 +423,10 @@
   </si>
   <si>
     <t>merge into</t>
+    <phoneticPr fontId="3" type="noConversion"/>
+  </si>
+  <si>
+    <t>6201; 6202</t>
     <phoneticPr fontId="3" type="noConversion"/>
   </si>
 </sst>
@@ -908,7 +909,7 @@
       </c>
       <c r="B1" s="14"/>
       <c r="C1" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
@@ -916,7 +917,7 @@
         <v>1</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="E2" s="12"/>
     </row>
@@ -973,7 +974,7 @@
         <v>6</v>
       </c>
       <c r="B7" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="E7" s="11"/>
     </row>
@@ -1015,7 +1016,7 @@
         <v>10</v>
       </c>
       <c r="B11" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="E11" s="12"/>
     </row>
@@ -1237,7 +1238,7 @@
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A31" s="4"/>
       <c r="B31" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="E31" s="12"/>
     </row>
@@ -1316,7 +1317,7 @@
         <v>58</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="E40" s="12"/>
     </row>
@@ -1506,7 +1507,7 @@
     </row>
     <row r="56" spans="1:11" x14ac:dyDescent="0.3">
       <c r="A56" s="8" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>93</v>
@@ -1579,7 +1580,7 @@
         <v>100</v>
       </c>
       <c r="B63" s="9" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C63" s="1"/>
       <c r="E63" s="12"/>
@@ -1589,55 +1590,55 @@
         <v>101</v>
       </c>
       <c r="B64" s="2" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="E64" s="12"/>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="2" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="B65" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="E65" s="12"/>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="6" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="B66" s="6" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C66" s="2" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="E66" s="12"/>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="6" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="B67" s="6" t="s">
-        <v>110</v>
+        <v>109</v>
       </c>
       <c r="C67" s="2" t="s">
-        <v>102</v>
+        <v>127</v>
       </c>
       <c r="E67" s="12"/>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A68" s="3" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B68" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="E68" s="12"/>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="13" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="B69" s="14"/>
       <c r="D69">
@@ -1647,40 +1648,40 @@
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A70" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="E70" s="12"/>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B71" s="2" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="E71" s="12"/>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="6" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B72" s="6" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="C72" s="2" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E72" s="12"/>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A73" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B73" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D73">
         <v>6</v>

</xml_diff>